<commit_message>
Highlight disabled buttons by retaining purple gradient
</commit_message>
<xml_diff>
--- a/backend/candidates_16612688-3635-4101-a28f-3209733a2249.xlsx
+++ b/backend/candidates_16612688-3635-4101-a28f-3209733a2249.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1243"/>
+  <dimension ref="A1:G1244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46347,6 +46347,43 @@
         </is>
       </c>
     </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>bd190710-98d6-4f19-87de-4fee43661501</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Tumul</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>tumul@example.com</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>65.0%</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>2026-08-31 12:34:36</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>